<commit_message>
Four column CGST, SGST and other two related column added in PO Import template
</commit_message>
<xml_diff>
--- a/public/templates/PO Upload Template.xlsx
+++ b/public/templates/PO Upload Template.xlsx
@@ -616,9 +616,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AK10"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" customWidth="1"/>
@@ -641,20 +641,21 @@
     <col min="20" max="20" width="26.28515625" customWidth="1"/>
     <col min="21" max="21" width="9.7109375" customWidth="1"/>
     <col min="22" max="22" width="18.42578125" customWidth="1"/>
-    <col min="23" max="23" width="18" customWidth="1"/>
-    <col min="24" max="24" width="26.7109375" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" customWidth="1"/>
-    <col min="26" max="26" width="18.85546875" customWidth="1"/>
-    <col min="27" max="27" width="18.5703125" customWidth="1"/>
-    <col min="28" max="28" width="27.28515625" customWidth="1"/>
-    <col min="29" max="29" width="18" customWidth="1"/>
-    <col min="30" max="30" width="26.7109375" customWidth="1"/>
+    <col min="23" max="26" width="25" customWidth="1"/>
+    <col min="27" max="27" width="18" customWidth="1"/>
+    <col min="28" max="28" width="26.7109375" customWidth="1"/>
+    <col min="29" max="29" width="10.140625" customWidth="1"/>
+    <col min="30" max="30" width="18.85546875" customWidth="1"/>
     <col min="31" max="31" width="18.5703125" customWidth="1"/>
     <col min="32" max="32" width="27.28515625" customWidth="1"/>
-    <col min="33" max="33" width="20.140625" customWidth="1"/>
+    <col min="33" max="33" width="18" customWidth="1"/>
+    <col min="34" max="34" width="26.7109375" customWidth="1"/>
+    <col min="35" max="35" width="18.5703125" customWidth="1"/>
+    <col min="36" max="36" width="27.28515625" customWidth="1"/>
+    <col min="37" max="37" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" ht="32.1" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -666,7 +667,7 @@
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:33" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:33" ht="21.75" ns3:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -691,7 +692,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:33" ht="21.75" ns3:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -706,7 +707,7 @@
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
     </row>
-    <row r="4" spans="1:33" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:33" ht="21.75" ns3:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -725,7 +726,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:33" ht="43.5" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:33" ht="43.5" ns3:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -740,7 +741,7 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:33" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:33" ht="21.75" ns3:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -759,7 +760,7 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:33" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:33" ht="21.75" ns3:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -774,8 +775,8 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:33" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" ht="15" customHeight="1" ns3:dyDescent="0.25"/>
+    <row r="9" spans="1:33" ht="43.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -842,41 +843,53 @@
       <c r="V9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="W9" s="3" t="s">
+      <c r="W9" s="3" t="str">
+        <v>Buying Tax CGST</v>
+      </c>
+      <c r="X9" s="3" t="str">
+        <v>Buying Tax CGST Amount</v>
+      </c>
+      <c r="Y9" s="3" t="str">
+        <v>Buying Tax SGST</v>
+      </c>
+      <c r="Z9" s="3" t="str">
+        <v>Buying Tax SGST Amount</v>
+      </c>
+      <c r="AA9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="X9" s="3" t="s">
+      <c r="AB9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="Y9" s="3" t="s">
+      <c r="AC9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Z9" s="3" t="s">
+      <c r="AD9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AA9" s="3" t="s">
+      <c r="AE9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AB9" s="3" t="s">
+      <c r="AF9" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="AC9" s="3" t="s">
+      <c r="AG9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="AD9" s="3" t="s">
+      <c r="AH9" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AE9" s="3" t="s">
+      <c r="AI9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="AF9" s="3" t="s">
+      <c r="AJ9" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="AG9" s="4" t="s">
+      <c r="AK9" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:33" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" ht="43.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A10" s="5">
         <v>94199992</v>
       </c>
@@ -939,23 +952,23 @@
       <c r="V10" s="6">
         <v>0</v>
       </c>
-      <c r="W10" s="6">
+      <c r="W10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="6">
         <v>18</v>
       </c>
-      <c r="X10" s="6">
+      <c r="AB10" s="6">
         <v>198.36</v>
-      </c>
-      <c r="Y10" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="6">
-        <v>9</v>
-      </c>
-      <c r="AB10" s="6">
-        <v>625.35</v>
       </c>
       <c r="AC10" s="6">
         <v>0</v>
@@ -969,7 +982,19 @@
       <c r="AF10" s="6">
         <v>625.35</v>
       </c>
-      <c r="AG10" s="7" t="s">
+      <c r="AG10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="6">
+        <v>9</v>
+      </c>
+      <c r="AJ10" s="6">
+        <v>625.35</v>
+      </c>
+      <c r="AK10" s="7" t="s">
         <v>58</v>
       </c>
     </row>
@@ -990,7 +1015,7 @@
     <mergeCell ref="E6:I7"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="AG10:AG1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="AK10:AK1000" ns2:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"SuitCase,BackPack,Small Hard Case"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>